<commit_message>
Let a topic say what a positive position means
Continuum 1 runs from Oppose to Support, which tells a reader nothing
until the page says what a positive position on this topic is. Topics
gain an axis column that supplies that line; a topic with none prints
no line rather than a guess. The column rides through the workbook,
the CSVs and the four exports.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KjnsA5EXCtANSJ7uyuepXy
</commit_message>
<xml_diff>
--- a/tools/static-site/ISE_Data_Entry.xlsx
+++ b/tools/static-site/ISE_Data_Entry.xlsx
@@ -15,7 +15,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'pages'!$A$1:$AC$262</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'edges'!$A$1:$T$898</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'topics'!$A$1:$E$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'topics'!$A$1:$F$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,6 +455,11 @@
         <t>topic: what sits inside this page and what belongs to a neighbouring topic with its own page.</t>
       </text>
     </comment>
+    <comment ref="F1" authorId="0" shapeId="0">
+      <text>
+        <t>topic: what a positive position means on this topic and what a negative one means, so a reader can place a belief on Continuum 1 without guessing. Blank means the site says only Oppose and Support.</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
@@ -31926,7 +31931,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E79"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -31934,6 +31939,7 @@
     <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -31962,6 +31968,11 @@
           <t>scope</t>
         </is>
       </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>axis</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -33310,7 +33321,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E79"/>
+  <autoFilter ref="A1:F79"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>

<commit_message>
Add the engagement cells of the ethics topic page and two debates on psychology
Seven engagement rows and eight more rungs on the public office topic,
each drafted from the beliefs beneath it and checked against them, and
the Psychology sub-topic's definition, axis and two argued beliefs.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KjnsA5EXCtANSJ7uyuepXy
</commit_message>
<xml_diff>
--- a/tools/static-site/ISE_Data_Entry.xlsx
+++ b/tools/static-site/ISE_Data_Entry.xlsx
@@ -13,8 +13,8 @@
     <sheet name="topics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'pages'!$A$1:$AC$402</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'edges'!$A$1:$T$1058</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'pages'!$A$1:$AC$416</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'edges'!$A$1:$T$1085</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'topics'!$A$1:$F$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -859,7 +859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC402"/>
+  <dimension ref="A1:AC416"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -13967,8 +13967,342 @@
         </is>
       </c>
     </row>
+    <row r="403">
+      <c r="A403" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+      <c r="C403" s="5" t="inlineStr">
+        <is>
+          <t>belief</t>
+        </is>
+      </c>
+      <c r="D403" s="4" t="inlineStr">
+        <is>
+          <t>Most people with depression or anxiety would clearly benefit from professional treatment rather than handling it on their own.</t>
+        </is>
+      </c>
+      <c r="F403" s="5" t="inlineStr">
+        <is>
+          <t>psychology</t>
+        </is>
+      </c>
+      <c r="W403" s="4" t="inlineStr">
+        <is>
+          <t>The disagreement turns on whether common sadness and worry are illnesses that need expert care or ordinary struggles that most people can and should work through themselves.</t>
+        </is>
+      </c>
+      <c r="AA403" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="AB403" s="5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="4" t="inlineStr">
+        <is>
+          <t>trained-therapists-doctors-have</t>
+        </is>
+      </c>
+      <c r="C404" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D404" s="4" t="inlineStr">
+        <is>
+          <t>Trained therapists and doctors have methods that work and that a person cannot easily apply to themselves, just as a person cannot set their own broken bone well.</t>
+        </is>
+      </c>
+      <c r="G404" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="4" t="inlineStr">
+        <is>
+          <t>very-symptoms-depression-low</t>
+        </is>
+      </c>
+      <c r="C405" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D405" s="4" t="inlineStr">
+        <is>
+          <t>The very symptoms of depression, low energy and hopelessness, make self-help unlikely to succeed, because the illness attacks the will needed to fight it.</t>
+        </is>
+      </c>
+      <c r="G405" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="4" t="inlineStr">
+        <is>
+          <t>untreated-problems-tend-grow</t>
+        </is>
+      </c>
+      <c r="C406" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D406" s="4" t="inlineStr">
+        <is>
+          <t>Untreated problems tend to grow, affecting work, family, and physical health, so early professional care prevents larger costs later.</t>
+        </is>
+      </c>
+      <c r="G406" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="4" t="inlineStr">
+        <is>
+          <t>sadness-worry-normal-responses</t>
+        </is>
+      </c>
+      <c r="C407" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D407" s="4" t="inlineStr">
+        <is>
+          <t>Sadness and worry are normal responses to hard lives, and calling them illnesses teaches people they are broken when they are simply struggling.</t>
+        </is>
+      </c>
+      <c r="G407" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="4" t="inlineStr">
+        <is>
+          <t>many-people-recover-fully</t>
+        </is>
+      </c>
+      <c r="C408" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D408" s="4" t="inlineStr">
+        <is>
+          <t>Many people recover fully through exercise, sleep, friendship, and time, and steering them all toward clinics uses up limited care that the severely ill need.</t>
+        </is>
+      </c>
+      <c r="G408" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="4" t="inlineStr">
+        <is>
+          <t>treatment-carries-its-own</t>
+        </is>
+      </c>
+      <c r="C409" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D409" s="4" t="inlineStr">
+        <is>
+          <t>Treatment carries its own risks, including medication side effects and dependence on a therapist, that are worth accepting only when the problem is serious.</t>
+        </is>
+      </c>
+      <c r="G409" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+      <c r="C410" s="5" t="inlineStr">
+        <is>
+          <t>belief</t>
+        </is>
+      </c>
+      <c r="D410" s="4" t="inlineStr">
+        <is>
+          <t>Teaching children to build toughness and tolerate discomfort does more for their mental health than teaching them to monitor and talk about their feelings.</t>
+        </is>
+      </c>
+      <c r="F410" s="5" t="inlineStr">
+        <is>
+          <t>psychology</t>
+        </is>
+      </c>
+      <c r="W410" s="4" t="inlineStr">
+        <is>
+          <t>The disagreement turns on whether paying close attention to feelings makes children stronger by helping them ask for help or weaker by making small worries loom large.</t>
+        </is>
+      </c>
+      <c r="AA410" s="5" t="n">
+        <v>-45</v>
+      </c>
+      <c r="AB410" s="5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="4" t="inlineStr">
+        <is>
+          <t>constant-attention-feelings-can</t>
+        </is>
+      </c>
+      <c r="C411" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D411" s="4" t="inlineStr">
+        <is>
+          <t>Constant attention to feelings can make small worries seem large, and children who learn to push through discomfort discover they can handle more than they feared.</t>
+        </is>
+      </c>
+      <c r="G411" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="4" t="inlineStr">
+        <is>
+          <t>life-will-bring-hardship</t>
+        </is>
+      </c>
+      <c r="C412" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D412" s="4" t="inlineStr">
+        <is>
+          <t>Life will bring hardship that no amount of talking can prevent, so the skill that lasts is the ability to keep going through it.</t>
+        </is>
+      </c>
+      <c r="G412" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="4" t="inlineStr">
+        <is>
+          <t>children-who-treated-fragile</t>
+        </is>
+      </c>
+      <c r="C413" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D413" s="4" t="inlineStr">
+        <is>
+          <t>Children who are treated as fragile tend to act fragile, while children expected to cope generally rise to the expectation.</t>
+        </is>
+      </c>
+      <c r="G413" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="4" t="inlineStr">
+        <is>
+          <t>children-who-cannot-name</t>
+        </is>
+      </c>
+      <c r="C414" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D414" s="4" t="inlineStr">
+        <is>
+          <t>Children who cannot name what they feel cannot ask for help, and telling them to tough it out teaches them to hide problems until they become crises.</t>
+        </is>
+      </c>
+      <c r="G414" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="4" t="inlineStr">
+        <is>
+          <t>toughness-training-works-children</t>
+        </is>
+      </c>
+      <c r="C415" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D415" s="4" t="inlineStr">
+        <is>
+          <t>Toughness training works for children who are already secure, but for a child who is being bullied or abused it means suffering in silence.</t>
+        </is>
+      </c>
+      <c r="G415" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="4" t="inlineStr">
+        <is>
+          <t>talking-about-feelings-building</t>
+        </is>
+      </c>
+      <c r="C416" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D416" s="4" t="inlineStr">
+        <is>
+          <t>Talking about feelings and building toughness are not opposites; naming a fear is often the first step to facing it.</t>
+        </is>
+      </c>
+      <c r="G416" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AC402"/>
+  <autoFilter ref="A1:AC416"/>
   <dataValidations count="5">
     <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"belief,claim,linkage,importance,interest,uniqueness,equivalence,driver,media"</formula1>
@@ -13997,7 +14331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1058"/>
+  <dimension ref="A1:T1085"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -39010,8 +39344,712 @@
         </is>
       </c>
     </row>
+    <row r="1059">
+      <c r="A1059" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1059" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1059" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1059" s="4" t="inlineStr">
+        <is>
+          <t>clemency-only-executive-power</t>
+        </is>
+      </c>
+      <c r="O1059" s="4" t="inlineStr">
+        <is>
+          <t>D.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1060" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1060" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1060" s="4" t="inlineStr">
+        <is>
+          <t>article-ii-grants-power</t>
+        </is>
+      </c>
+      <c r="O1060" s="4" t="inlineStr">
+        <is>
+          <t>D.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1061" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1061" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1061" s="4" t="inlineStr">
+        <is>
+          <t>pardons-granted-president-s</t>
+        </is>
+      </c>
+      <c r="O1061" s="4" t="inlineStr">
+        <is>
+          <t>D.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1062" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1062" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1062" s="4" t="inlineStr">
+        <is>
+          <t>narrower-fix-reaches-actual</t>
+        </is>
+      </c>
+      <c r="O1062" s="4" t="inlineStr">
+        <is>
+          <t>D.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1063" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1063" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1063" s="4" t="inlineStr">
+        <is>
+          <t>two-thirds-threshold-means</t>
+        </is>
+      </c>
+      <c r="O1063" s="4" t="inlineStr">
+        <is>
+          <t>D.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1064" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1064" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1064" s="4" t="inlineStr">
+        <is>
+          <t>clemency-exists-correct-injustices</t>
+        </is>
+      </c>
+      <c r="O1064" s="4" t="inlineStr">
+        <is>
+          <t>D.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1065" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1065" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1065" s="4" t="inlineStr">
+        <is>
+          <t>most-states-already-put</t>
+        </is>
+      </c>
+      <c r="O1065" s="4" t="inlineStr">
+        <is>
+          <t>D.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1066" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1066" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1066" s="4" t="inlineStr">
+        <is>
+          <t>reversible-pardon-pardon-nobody</t>
+        </is>
+      </c>
+      <c r="O1066" s="4" t="inlineStr">
+        <is>
+          <t>D.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1067" s="5" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="C1067" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="E1067" s="4" t="inlineStr">
+        <is>
+          <t>A voter who thinks members of Congress should not trade the stocks of industries their committees oversee, votes for candidates who say so when the choice is easy, and otherwise leaves the matter alone.</t>
+        </is>
+      </c>
+      <c r="O1067" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T1067" s="4" t="inlineStr">
+        <is>
+          <t>example: sympathetic voter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1068" s="5" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="C1068" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="E1068" s="4" t="inlineStr">
+        <is>
+          <t>A voter who believes the disclosure form and the existing conflict-of-interest statutes already catch what matters, doubts a new ban would deter anyone but honest people of ordinary means, and says so only when asked.</t>
+        </is>
+      </c>
+      <c r="O1068" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="T1068" s="4" t="inlineStr">
+        <is>
+          <t>example: skeptical voter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1069" s="5" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="C1069" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="E1069" s="4" t="inlineStr">
+        <is>
+          <t>A citizen who writes to their representative to demand a vote on the drafted holdings ban, signs and circulates petitions, backs candidates who pledge not to trade individual stocks, and asks publicly why the Senate has not scheduled the vote.</t>
+        </is>
+      </c>
+      <c r="O1069" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="T1069" s="4" t="inlineStr">
+        <is>
+          <t>example: reform campaigner</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1070" s="5" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="C1070" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="E1070" s="4" t="inlineStr">
+        <is>
+          <t>A citizen or former official who testifies, writes and organizes against new bans, argues that forced divestiture narrows who can afford to serve and reaches spouses and children who never ran, and pushes instead to strengthen the disclosure form and the audits.</t>
+        </is>
+      </c>
+      <c r="O1070" s="4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="T1070" s="4" t="inlineStr">
+        <is>
+          <t>example: disclosure-first advocate</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1071" s="5" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="C1071" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="E1071" s="4" t="inlineStr">
+        <is>
+          <t>An officeholder who sells their individual stocks or moves them into a blind trust, publishes their own tax returns, and declines to give any official role to a relative, all without a rule requiring it, while leaving colleagues to make their own choice.</t>
+        </is>
+      </c>
+      <c r="O1071" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T1071" s="4" t="inlineStr">
+        <is>
+          <t>example: self-divesting officeholder</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1072" s="5" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="C1072" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="E1072" s="4" t="inlineStr">
+        <is>
+          <t>An officeholder who keeps lawful individual holdings, refuses to sign a voluntary pledge to divest or to publish returns, states plainly that the law does not require it and that officials keep the ordinary rights of citizens, and does not try to stop others from pledging.</t>
+        </is>
+      </c>
+      <c r="O1072" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="T1072" s="4" t="inlineStr">
+        <is>
+          <t>example: pledge-declining officeholder</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1073" s="5" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="C1073" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="E1073" s="4" t="inlineStr">
+        <is>
+          <t>A person with lawful access to an official's confidential tax return who publishes it under their own name to show what the disclosure form leaves out, knowing the law attaches criminal penalties to unauthorized disclosure, and accepts prosecution as the price of forcing the question.</t>
+        </is>
+      </c>
+      <c r="O1073" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="T1073" s="4" t="inlineStr">
+        <is>
+          <t>example: open-disclosure lawbreaker</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+      <c r="B1074" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1074" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1074" s="4" t="inlineStr">
+        <is>
+          <t>trained-therapists-doctors-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+      <c r="B1075" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1075" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1075" s="4" t="inlineStr">
+        <is>
+          <t>very-symptoms-depression-low</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+      <c r="B1076" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1076" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1076" s="4" t="inlineStr">
+        <is>
+          <t>untreated-problems-tend-grow</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+      <c r="B1077" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1077" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1077" s="4" t="inlineStr">
+        <is>
+          <t>sadness-worry-normal-responses</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+      <c r="B1078" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1078" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1078" s="4" t="inlineStr">
+        <is>
+          <t>many-people-recover-fully</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="4" t="inlineStr">
+        <is>
+          <t>most-people-depression-anxiety</t>
+        </is>
+      </c>
+      <c r="B1079" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1079" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1079" s="4" t="inlineStr">
+        <is>
+          <t>treatment-carries-its-own</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+      <c r="B1080" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1080" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1080" s="4" t="inlineStr">
+        <is>
+          <t>constant-attention-feelings-can</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+      <c r="B1081" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1081" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1081" s="4" t="inlineStr">
+        <is>
+          <t>life-will-bring-hardship</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+      <c r="B1082" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1082" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1082" s="4" t="inlineStr">
+        <is>
+          <t>children-who-treated-fragile</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+      <c r="B1083" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1083" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1083" s="4" t="inlineStr">
+        <is>
+          <t>children-who-cannot-name</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+      <c r="B1084" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1084" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1084" s="4" t="inlineStr">
+        <is>
+          <t>toughness-training-works-children</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="4" t="inlineStr">
+        <is>
+          <t>teaching-children-build-toughness</t>
+        </is>
+      </c>
+      <c r="B1085" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1085" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1085" s="4" t="inlineStr">
+        <is>
+          <t>talking-about-feelings-building</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T1058"/>
+  <autoFilter ref="A1:T1085"/>
   <dataValidations count="2">
     <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"argument,assumption,bias,category,cba,common,component,compromise,criteria,criterion,definition,direction,dispute,downstream,engagement,evidence,falsify,impact,interest,interest_listing,law,long_term,media,motive,obstacle,person,prediction,related,rung,shared_interest,short_term,similar,stack,strength,topic_media,topic_values,upstream,value"</formula1>
@@ -40417,6 +41455,16 @@
           <t>social-science</t>
         </is>
       </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>How the mind works, why people feel and act as they do, and how mental health problems are understood and treated.</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>favors treating mental struggles as medical conditions best handled by professionals and treatment; negative favors seeing them as ordinary parts of life best handled through relationships, habits, and personal effort.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Import the first wiki position and three more sub-topics' debates
"We should support and strengthen democracy to restore the voter's
voice" comes over from the wiki with its five reasons each way, eight
cited findings and the interests on both sides, filed under a new
Democracy & Rule of Law topic. The other five group topics the wiki
sidebar names (Core Principles, Rights & Liberty, Evidence & Process,
Energy, Immigration) get their pages now so the remaining imports have
somewhere to land. Internet, Jobs and Trade each get a definition, an
axis and two argued beliefs; the ethics topic page gains its Objective
Criteria and Related Topics rows.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KjnsA5EXCtANSJ7uyuepXy
</commit_message>
<xml_diff>
--- a/tools/static-site/ISE_Data_Entry.xlsx
+++ b/tools/static-site/ISE_Data_Entry.xlsx
@@ -13,9 +13,9 @@
     <sheet name="topics" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'pages'!$A$1:$AC$416</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'edges'!$A$1:$T$1085</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'topics'!$A$1:$F$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'pages'!$A$1:$AC$490</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'edges'!$A$1:$T$1166</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'topics'!$A$1:$F$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -859,7 +859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC416"/>
+  <dimension ref="A1:AC490"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14301,8 +14301,1717 @@
         </is>
       </c>
     </row>
+    <row r="417">
+      <c r="A417" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+      <c r="C417" s="5" t="inlineStr">
+        <is>
+          <t>belief</t>
+        </is>
+      </c>
+      <c r="D417" s="4" t="inlineStr">
+        <is>
+          <t>Tariffs on imported goods generally cost a country's consumers more than they save its workers.</t>
+        </is>
+      </c>
+      <c r="F417" s="5" t="inlineStr">
+        <is>
+          <t>trade</t>
+        </is>
+      </c>
+      <c r="W417" s="4" t="inlineStr">
+        <is>
+          <t>Whether a small cost spread across everyone is worse than a large cost concentrated on the towns and workers who lose.</t>
+        </is>
+      </c>
+      <c r="AA417" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="AB417" s="5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="4" t="inlineStr">
+        <is>
+          <t>tariff-raises-price-good</t>
+        </is>
+      </c>
+      <c r="C418" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D418" s="4" t="inlineStr">
+        <is>
+          <t>A tariff raises the price of the good for every buyer in the country, while it protects only the workers in one industry.</t>
+        </is>
+      </c>
+      <c r="G418" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="4" t="inlineStr">
+        <is>
+          <t>other-countries-answer-tariffs</t>
+        </is>
+      </c>
+      <c r="C419" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D419" s="4" t="inlineStr">
+        <is>
+          <t>Other countries answer tariffs with their own, so exporters in industries that were never in trouble lose their foreign customers.</t>
+        </is>
+      </c>
+      <c r="G419" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="4" t="inlineStr">
+        <is>
+          <t>industries-shielded-foreign-competition</t>
+        </is>
+      </c>
+      <c r="C420" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D420" s="4" t="inlineStr">
+        <is>
+          <t>Industries shielded from foreign competition tend to stop improving, so the country ends up paying more for worse products.</t>
+        </is>
+      </c>
+      <c r="G420" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="4" t="inlineStr">
+        <is>
+          <t>when-factory-closes-whole</t>
+        </is>
+      </c>
+      <c r="C421" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D421" s="4" t="inlineStr">
+        <is>
+          <t>When a factory closes, a whole town can lose its tax base, its shops and its future, and that damage is far larger than a small price increase spread across everyone.</t>
+        </is>
+      </c>
+      <c r="G421" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="4" t="inlineStr">
+        <is>
+          <t>when-tariff-removed-importers</t>
+        </is>
+      </c>
+      <c r="C422" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D422" s="4" t="inlineStr">
+        <is>
+          <t>When a tariff is removed, importers and retailers often keep much of the price difference for themselves rather than passing it on, so the saving that reaches shoppers is smaller than the wages that were lost.</t>
+        </is>
+      </c>
+      <c r="G422" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="4" t="inlineStr">
+        <is>
+          <t>country-lets-its-factories</t>
+        </is>
+      </c>
+      <c r="C423" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D423" s="4" t="inlineStr">
+        <is>
+          <t>A country that lets its factories die loses the skills and supply chains it would need in a war or a crisis, and no price saving is worth that.</t>
+        </is>
+      </c>
+      <c r="G423" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+      <c r="C424" s="5" t="inlineStr">
+        <is>
+          <t>belief</t>
+        </is>
+      </c>
+      <c r="D424" s="4" t="inlineStr">
+        <is>
+          <t>A country should protect its key manufacturing industries with tariffs even when imports are cheaper.</t>
+        </is>
+      </c>
+      <c r="F424" s="5" t="inlineStr">
+        <is>
+          <t>trade</t>
+        </is>
+      </c>
+      <c r="W424" s="4" t="inlineStr">
+        <is>
+          <t>Whether the goods a country cannot afford to lose can be identified honestly and protected more cheaply than with a tariff.</t>
+        </is>
+      </c>
+      <c r="AA424" s="5" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AB424" s="5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="4" t="inlineStr">
+        <is>
+          <t>country-cannot-make-its</t>
+        </is>
+      </c>
+      <c r="C425" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D425" s="4" t="inlineStr">
+        <is>
+          <t>A country that cannot make its own steel, chips or medicine is at the mercy of whoever does, and that is a matter of security rather than price.</t>
+        </is>
+      </c>
+      <c r="G425" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="4" t="inlineStr">
+        <is>
+          <t>manufacturing-jobs-offer-steady</t>
+        </is>
+      </c>
+      <c r="C426" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D426" s="4" t="inlineStr">
+        <is>
+          <t>Manufacturing jobs offer steady middle-class pay to people without college degrees in a way that few service jobs do.</t>
+        </is>
+      </c>
+      <c r="G426" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="4" t="inlineStr">
+        <is>
+          <t>new-industries-need-time</t>
+        </is>
+      </c>
+      <c r="C427" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D427" s="4" t="inlineStr">
+        <is>
+          <t>New industries need time to grow before they can compete with established foreign rivals, and a tariff buys that time.</t>
+        </is>
+      </c>
+      <c r="G427" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="4" t="inlineStr">
+        <is>
+          <t>every-industry-calls-itself</t>
+        </is>
+      </c>
+      <c r="C428" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D428" s="4" t="inlineStr">
+        <is>
+          <t>Every industry calls itself key when a tariff is on offer, so protection ends up going to whoever lobbies hardest rather than to what a country truly needs.</t>
+        </is>
+      </c>
+      <c r="G428" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="4" t="inlineStr">
+        <is>
+          <t>manufacturers-who-use-protected</t>
+        </is>
+      </c>
+      <c r="C429" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D429" s="4" t="inlineStr">
+        <is>
+          <t>Manufacturers who use the protected good as an input pay more, so protecting one industry weakens the ones that depend on it.</t>
+        </is>
+      </c>
+      <c r="G429" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="4" t="inlineStr">
+        <is>
+          <t>country-wants-secure-supply</t>
+        </is>
+      </c>
+      <c r="C430" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D430" s="4" t="inlineStr">
+        <is>
+          <t>A country that wants secure supply can stockpile goods or fund a few plants directly, which costs far less than taxing every buyer.</t>
+        </is>
+      </c>
+      <c r="G430" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+      <c r="C431" s="5" t="inlineStr">
+        <is>
+          <t>belief</t>
+        </is>
+      </c>
+      <c r="D431" s="4" t="inlineStr">
+        <is>
+          <t>Raising the minimum wage generally helps low-paid workers more than it hurts them.</t>
+        </is>
+      </c>
+      <c r="F431" s="5" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="W431" s="4" t="inlineStr">
+        <is>
+          <t>Whether employers respond to a higher wage floor mostly by paying more or mostly by hiring less.</t>
+        </is>
+      </c>
+      <c r="AA431" s="5" t="n">
+        <v>55</v>
+      </c>
+      <c r="AB431" s="5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="4" t="inlineStr">
+        <is>
+          <t>single-worker-has-almost</t>
+        </is>
+      </c>
+      <c r="C432" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D432" s="4" t="inlineStr">
+        <is>
+          <t>A single worker has almost no power to bargain with a large employer, and a wage floor gives them the bargaining position they lack.</t>
+        </is>
+      </c>
+      <c r="G432" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="4" t="inlineStr">
+        <is>
+          <t>low-paid-workers-spend</t>
+        </is>
+      </c>
+      <c r="C433" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D433" s="4" t="inlineStr">
+        <is>
+          <t>Low-paid workers spend nearly everything they earn, so higher wages flow straight back into local businesses.</t>
+        </is>
+      </c>
+      <c r="G433" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="4" t="inlineStr">
+        <is>
+          <t>when-wages-too-low</t>
+        </is>
+      </c>
+      <c r="C434" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D434" s="4" t="inlineStr">
+        <is>
+          <t>When wages are too low to live on, taxpayers end up topping them up through public benefits, which is a subsidy to low-paying employers.</t>
+        </is>
+      </c>
+      <c r="G434" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="4" t="inlineStr">
+        <is>
+          <t>when-labor-costs-more</t>
+        </is>
+      </c>
+      <c r="C435" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D435" s="4" t="inlineStr">
+        <is>
+          <t>When labor costs more, employers hire fewer people, cut hours or turn to machines, and the workers who lose out are the least skilled.</t>
+        </is>
+      </c>
+      <c r="G435" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="4" t="inlineStr">
+        <is>
+          <t>small-businesses-poorer-regions</t>
+        </is>
+      </c>
+      <c r="C436" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D436" s="4" t="inlineStr">
+        <is>
+          <t>Small businesses in poorer regions cannot pay what a big-city employer can, so one national floor destroys jobs where they are most needed.</t>
+        </is>
+      </c>
+      <c r="G436" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="4" t="inlineStr">
+        <is>
+          <t>many-minimum-wage-earners</t>
+        </is>
+      </c>
+      <c r="C437" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D437" s="4" t="inlineStr">
+        <is>
+          <t>Many minimum-wage earners are young people or second earners in comfortable households, so a higher minimum wage misses the poorest families it is meant to help.</t>
+        </is>
+      </c>
+      <c r="G437" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+      <c r="C438" s="5" t="inlineStr">
+        <is>
+          <t>belief</t>
+        </is>
+      </c>
+      <c r="D438" s="4" t="inlineStr">
+        <is>
+          <t>Employers should generally be free to fire workers without having to show a reason, as long as the firing is not discriminatory.</t>
+        </is>
+      </c>
+      <c r="F438" s="5" t="inlineStr">
+        <is>
+          <t>jobs</t>
+        </is>
+      </c>
+      <c r="W438" s="4" t="inlineStr">
+        <is>
+          <t>Whether making firing easy creates more jobs than it makes worse.</t>
+        </is>
+      </c>
+      <c r="AA438" s="5" t="n">
+        <v>-55</v>
+      </c>
+      <c r="AB438" s="5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="4" t="inlineStr">
+        <is>
+          <t>employer-who-knows-firing</t>
+        </is>
+      </c>
+      <c r="C439" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D439" s="4" t="inlineStr">
+        <is>
+          <t>An employer who knows firing will be hard is slower to hire in the first place, so strict rules protect people who have jobs at the expense of people who want them.</t>
+        </is>
+      </c>
+      <c r="G439" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="4" t="inlineStr">
+        <is>
+          <t>small-businesses-cannot-afford</t>
+        </is>
+      </c>
+      <c r="C440" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D440" s="4" t="inlineStr">
+        <is>
+          <t>Small businesses cannot afford the lawyers and paperwork needed to build a case for every dismissal.</t>
+        </is>
+      </c>
+      <c r="G440" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="4" t="inlineStr">
+        <is>
+          <t>workers-can-quit-job</t>
+        </is>
+      </c>
+      <c r="C441" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D441" s="4" t="inlineStr">
+        <is>
+          <t>Workers can quit a job without giving a reason, so fairness requires that employers be able to end the same working relationship without giving one.</t>
+        </is>
+      </c>
+      <c r="G441" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="4" t="inlineStr">
+        <is>
+          <t>losing-job-can-mean</t>
+        </is>
+      </c>
+      <c r="C442" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D442" s="4" t="inlineStr">
+        <is>
+          <t>Losing a job can mean losing a home, health coverage and a family's stability, and something that serious should require a reason.</t>
+        </is>
+      </c>
+      <c r="G442" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="4" t="inlineStr">
+        <is>
+          <t>workers-who-can-fired</t>
+        </is>
+      </c>
+      <c r="C443" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D443" s="4" t="inlineStr">
+        <is>
+          <t>Workers who can be fired at any moment are afraid to report safety problems, harassment or fraud.</t>
+        </is>
+      </c>
+      <c r="G443" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="4" t="inlineStr">
+        <is>
+          <t>rules-against-unfair-dismissal</t>
+        </is>
+      </c>
+      <c r="C444" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D444" s="4" t="inlineStr">
+        <is>
+          <t>Rules against unfair dismissal push employers to hire more carefully and manage better, which improves the workplace for everyone.</t>
+        </is>
+      </c>
+      <c r="G444" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+      <c r="C445" s="5" t="inlineStr">
+        <is>
+          <t>belief</t>
+        </is>
+      </c>
+      <c r="D445" s="4" t="inlineStr">
+        <is>
+          <t>Internet providers should generally be barred by law from speeding up, slowing down or charging extra for particular websites and services.</t>
+        </is>
+      </c>
+      <c r="F445" s="5" t="inlineStr">
+        <is>
+          <t>internet</t>
+        </is>
+      </c>
+      <c r="W445" s="4" t="inlineStr">
+        <is>
+          <t>The disagreement turns on whether competition and public attention are enough to keep providers honest, or whether the lack of choice in home internet makes a legal rule necessary.</t>
+        </is>
+      </c>
+      <c r="AA445" s="5" t="n">
+        <v>60</v>
+      </c>
+      <c r="AB445" s="5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="4" t="inlineStr">
+        <is>
+          <t>provider-can-slow-down</t>
+        </is>
+      </c>
+      <c r="C446" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D446" s="4" t="inlineStr">
+        <is>
+          <t>A provider that can slow down or charge extra for certain traffic gains a veto over which websites and services succeed, and that power belongs with users, not with the company selling the connection.</t>
+        </is>
+      </c>
+      <c r="G446" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="4" t="inlineStr">
+        <is>
+          <t>many-households-have-little</t>
+        </is>
+      </c>
+      <c r="C447" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D447" s="4" t="inlineStr">
+        <is>
+          <t>Many households have little real choice of home internet provider, so competition alone cannot punish one that plays favorites.</t>
+        </is>
+      </c>
+      <c r="G447" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="4" t="inlineStr">
+        <is>
+          <t>new-services-start-small</t>
+        </is>
+      </c>
+      <c r="C448" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D448" s="4" t="inlineStr">
+        <is>
+          <t>New services start small and cannot pay for fast lanes, so a rule of equal treatment keeps the door open for the next useful idea.</t>
+        </is>
+      </c>
+      <c r="G448" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="4" t="inlineStr">
+        <is>
+          <t>all-traffic-alike-live</t>
+        </is>
+      </c>
+      <c r="C449" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D449" s="4" t="inlineStr">
+        <is>
+          <t>Not all traffic is alike; a live video call suffers far more from delay than a file download does, and a legal ban on favoring traffic turns sensible prioritizing into a legal risk.</t>
+        </is>
+      </c>
+      <c r="G449" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="4" t="inlineStr">
+        <is>
+          <t>building-faster-networks-costs</t>
+        </is>
+      </c>
+      <c r="C450" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D450" s="4" t="inlineStr">
+        <is>
+          <t>Building faster networks costs a great deal, and letting providers charge the services that send the most traffic for faster delivery helps pay for upgrades that all users share.</t>
+        </is>
+      </c>
+      <c r="G450" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="4" t="inlineStr">
+        <is>
+          <t>providers-rarely-block-throttle</t>
+        </is>
+      </c>
+      <c r="C451" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D451" s="4" t="inlineStr">
+        <is>
+          <t>Providers rarely block or throttle in practice because customers and the press notice quickly, so the rule solves a problem that mostly does not occur.</t>
+        </is>
+      </c>
+      <c r="G451" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+      <c r="C452" s="5" t="inlineStr">
+        <is>
+          <t>belief</t>
+        </is>
+      </c>
+      <c r="D452" s="4" t="inlineStr">
+        <is>
+          <t>Laws that require people to prove their age before using social media do more harm than good.</t>
+        </is>
+      </c>
+      <c r="F452" s="5" t="inlineStr">
+        <is>
+          <t>internet</t>
+        </is>
+      </c>
+      <c r="W452" s="4" t="inlineStr">
+        <is>
+          <t>The disagreement turns on whether the privacy and access costs of checking everyone's age outweigh the harm to children the checks are meant to prevent.</t>
+        </is>
+      </c>
+      <c r="AA452" s="5" t="n">
+        <v>-50</v>
+      </c>
+      <c r="AB452" s="5" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="4" t="inlineStr">
+        <is>
+          <t>proving-age-means-handing</t>
+        </is>
+      </c>
+      <c r="C453" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D453" s="4" t="inlineStr">
+        <is>
+          <t>Proving age means handing an ID or a face scan to a company or a middleman, which creates a new store of sensitive data that can leak or be misused.</t>
+        </is>
+      </c>
+      <c r="G453" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="4" t="inlineStr">
+        <is>
+          <t>teenagers-who-blocked-mainstream</t>
+        </is>
+      </c>
+      <c r="C454" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D454" s="4" t="inlineStr">
+        <is>
+          <t>Teenagers who are blocked from mainstream sites do not stop going online; they move to smaller, less moderated places where the risks are greater.</t>
+        </is>
+      </c>
+      <c r="G454" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="4" t="inlineStr">
+        <is>
+          <t>age-rules-set-law</t>
+        </is>
+      </c>
+      <c r="C455" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D455" s="4" t="inlineStr">
+        <is>
+          <t>Age rules set by law sweep in adults too, since everyone has to pass the same check, so a protection for minors becomes a barrier for all.</t>
+        </is>
+      </c>
+      <c r="G455" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="4" t="inlineStr">
+        <is>
+          <t>society-already-requires-proof</t>
+        </is>
+      </c>
+      <c r="C456" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D456" s="4" t="inlineStr">
+        <is>
+          <t>Society already requires proof of age for alcohol, gambling and driving, and there is no principled reason that products children use heavily and that are built to hold their attention should be exempt.</t>
+        </is>
+      </c>
+      <c r="G456" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="4" t="inlineStr">
+        <is>
+          <t>leaving-choice-parents-has</t>
+        </is>
+      </c>
+      <c r="C457" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D457" s="4" t="inlineStr">
+        <is>
+          <t>Leaving the choice to parents has not worked, because a child needs only one friend with an account to feel left out, and parents cannot supervise every hour.</t>
+        </is>
+      </c>
+      <c r="G457" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="4" t="inlineStr">
+        <is>
+          <t>companies-can-verify-age</t>
+        </is>
+      </c>
+      <c r="C458" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D458" s="4" t="inlineStr">
+        <is>
+          <t>Companies can verify age without keeping the underlying documents, but voluntary adoption has been patchy and inconsistent, which is why a uniform legal requirement is needed.</t>
+        </is>
+      </c>
+      <c r="G458" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="C459" s="5" t="inlineStr">
+        <is>
+          <t>belief</t>
+        </is>
+      </c>
+      <c r="D459" s="4" t="inlineStr">
+        <is>
+          <t>We should support and strengthen democracy to restore the voter's voice.</t>
+        </is>
+      </c>
+      <c r="F459" s="5" t="inlineStr">
+        <is>
+          <t>democracy-and-rule-of-law</t>
+        </is>
+      </c>
+      <c r="W459" s="4" t="inlineStr">
+        <is>
+          <t>The problem diagnosis is strong: current electoral rules let unrepresentative primary electorates pick the choices, let mapmakers pick their voters, and make candidates depend on a narrow donor class. The reform mechanisms are less certain, since each specific fix (ranked-choice voting, nonpartisan primaries, commissions, donor matching) has real supporting evidence and real implementation risks, so this belief is strongest as "fix the structures, state by state, and measure" and weakest as a blanket endorsement of any one mechanism.</t>
+        </is>
+      </c>
+      <c r="AA459" s="5" t="n">
+        <v>80</v>
+      </c>
+      <c r="AB459" s="5" t="inlineStr">
+        <is>
+          <t>Strong</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="4" t="inlineStr">
+        <is>
+          <t>partisan-primaries-let-small</t>
+        </is>
+      </c>
+      <c r="C460" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D460" s="4" t="inlineStr">
+        <is>
+          <t>Partisan primaries let a small and unrepresentative group of voters pick the choices everyone else gets in the general election.</t>
+        </is>
+      </c>
+      <c r="G460" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="4" t="inlineStr">
+        <is>
+          <t>gerrymandering-lets-legislators-choose</t>
+        </is>
+      </c>
+      <c r="C461" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D461" s="4" t="inlineStr">
+        <is>
+          <t>Gerrymandering lets legislators choose their voters instead of voters choosing their legislators.</t>
+        </is>
+      </c>
+      <c r="G461" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="4" t="inlineStr">
+        <is>
+          <t>ranked-choice-voting-produces</t>
+        </is>
+      </c>
+      <c r="C462" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D462" s="4" t="inlineStr">
+        <is>
+          <t>Ranked-choice voting produces winners with broader support and reduces negative campaigning.</t>
+        </is>
+      </c>
+      <c r="G462" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="4" t="inlineStr">
+        <is>
+          <t>campaign-finance-structures-make</t>
+        </is>
+      </c>
+      <c r="C463" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D463" s="4" t="inlineStr">
+        <is>
+          <t>Campaign finance structures make candidates dependent on a donor class whose interests differ from those of their constituents.</t>
+        </is>
+      </c>
+      <c r="G463" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="4" t="inlineStr">
+        <is>
+          <t>third-parties-independents-kept</t>
+        </is>
+      </c>
+      <c r="C464" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D464" s="4" t="inlineStr">
+        <is>
+          <t>Third parties and independents are kept out by structural election rules, not because they are unpopular.</t>
+        </is>
+      </c>
+      <c r="G464" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="4" t="inlineStr">
+        <is>
+          <t>specific-electoral-reforms-have</t>
+        </is>
+      </c>
+      <c r="C465" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D465" s="4" t="inlineStr">
+        <is>
+          <t>Specific electoral reforms have real implementation problems and unintended consequences.</t>
+        </is>
+      </c>
+      <c r="G465" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="4" t="inlineStr">
+        <is>
+          <t>two-party-system-has</t>
+        </is>
+      </c>
+      <c r="C466" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D466" s="4" t="inlineStr">
+        <is>
+          <t>The two-party system has stabilizing effects that alternative systems may not replicate.</t>
+        </is>
+      </c>
+      <c r="G466" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="4" t="inlineStr">
+        <is>
+          <t>restoring-voter-s-voice</t>
+        </is>
+      </c>
+      <c r="C467" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D467" s="4" t="inlineStr">
+        <is>
+          <t>Restoring the voter's voice assumes there is a single coherent will of the voters to restore, but on many issues public opinion contradicts itself.</t>
+        </is>
+      </c>
+      <c r="G467" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="4" t="inlineStr">
+        <is>
+          <t>campaign-finance-restrictions-collide</t>
+        </is>
+      </c>
+      <c r="C468" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D468" s="4" t="inlineStr">
+        <is>
+          <t>Campaign finance restrictions collide with the First Amendment's protection of political spending as speech.</t>
+        </is>
+      </c>
+      <c r="G468" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="4" t="inlineStr">
+        <is>
+          <t>nonpartisan-primaries-may-weaken</t>
+        </is>
+      </c>
+      <c r="C469" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D469" s="4" t="inlineStr">
+        <is>
+          <t>Nonpartisan primaries may weaken party accountability rather than strengthen the voter's voice.</t>
+        </is>
+      </c>
+      <c r="G469" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="4" t="inlineStr">
+        <is>
+          <t>congress-polls-15-25</t>
+        </is>
+      </c>
+      <c r="C470" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D470" s="4" t="inlineStr">
+        <is>
+          <t>Congress polls at 15 to 25 percent approval while incumbent reelection rates exceed 90 percent.</t>
+        </is>
+      </c>
+      <c r="G470" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="4" t="inlineStr">
+        <is>
+          <t>primary-voters-measure-significantly</t>
+        </is>
+      </c>
+      <c r="C471" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D471" s="4" t="inlineStr">
+        <is>
+          <t>Primary voters measure significantly more ideologically extreme than each party's general-election supporters.</t>
+        </is>
+      </c>
+      <c r="G471" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="4" t="inlineStr">
+        <is>
+          <t>americans-identifying-independents-reached</t>
+        </is>
+      </c>
+      <c r="C472" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D472" s="4" t="inlineStr">
+        <is>
+          <t>Americans identifying as independents reached 43 percent, more than either party, while remaining excluded from most primaries.</t>
+        </is>
+      </c>
+      <c r="G472" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="4" t="inlineStr">
+        <is>
+          <t>alaska-s-first-federal</t>
+        </is>
+      </c>
+      <c r="C473" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D473" s="4" t="inlineStr">
+        <is>
+          <t>Alaska's first federal ranked-choice election showed none of the predicted voter confusion and had normal ballot-completion rates.</t>
+        </is>
+      </c>
+      <c r="G473" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="4" t="inlineStr">
+        <is>
+          <t>independent-redistricting-commissions-arizona</t>
+        </is>
+      </c>
+      <c r="C474" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D474" s="4" t="inlineStr">
+        <is>
+          <t>Independent redistricting commissions in Arizona and California reduced safe seats by 15 to 20 percent compared with maps drawn by legislatures.</t>
+        </is>
+      </c>
+      <c r="G474" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="4" t="inlineStr">
+        <is>
+          <t>policy-outcomes-correlate-preferences</t>
+        </is>
+      </c>
+      <c r="C475" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D475" s="4" t="inlineStr">
+        <is>
+          <t>Policy outcomes correlate with the preferences of economic elites at far higher rates than with the preferences of the median voter.</t>
+        </is>
+      </c>
+      <c r="G475" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="4" t="inlineStr">
+        <is>
+          <t>burlington-vermont-adopted-ranked</t>
+        </is>
+      </c>
+      <c r="C476" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D476" s="4" t="inlineStr">
+        <is>
+          <t>Burlington, Vermont adopted ranked-choice voting and then repealed it after the candidate with the most first-choice votes lost, though scholars dispute whether the result was actually unfair under the rules.</t>
+        </is>
+      </c>
+      <c r="G476" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="4" t="inlineStr">
+        <is>
+          <t>evidence-whether-nonpartisan-primaries</t>
+        </is>
+      </c>
+      <c r="C477" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D477" s="4" t="inlineStr">
+        <is>
+          <t>The evidence on whether nonpartisan primaries actually moderate candidates is mixed.</t>
+        </is>
+      </c>
+      <c r="G477" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="4" t="inlineStr">
+        <is>
+          <t>independent-voters-about-43</t>
+        </is>
+      </c>
+      <c r="C478" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D478" s="4" t="inlineStr">
+        <is>
+          <t>Independent voters, about 43 percent of Americans, need a meaningful vote because they are locked out of primaries.</t>
+        </is>
+      </c>
+      <c r="M478" s="5" t="inlineStr">
+        <is>
+          <t>Political equality</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="4" t="inlineStr">
+        <is>
+          <t>voters-need-representatives-who</t>
+        </is>
+      </c>
+      <c r="C479" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D479" s="4" t="inlineStr">
+        <is>
+          <t>Voters need representatives who solve problems rather than perform for their base audiences.</t>
+        </is>
+      </c>
+      <c r="M479" s="5" t="inlineStr">
+        <is>
+          <t>Accountability</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="4" t="inlineStr">
+        <is>
+          <t>forward-party-other-third</t>
+        </is>
+      </c>
+      <c r="C480" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D480" s="4" t="inlineStr">
+        <is>
+          <t>The Forward Party and other third parties need open primaries and ranked-choice rules because they benefit directly from them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="4" t="inlineStr">
+        <is>
+          <t>opponents-need-governmental-stability</t>
+        </is>
+      </c>
+      <c r="C481" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D481" s="4" t="inlineStr">
+        <is>
+          <t>Opponents need governmental stability and coherent governing coalitions.</t>
+        </is>
+      </c>
+      <c r="M481" s="5" t="inlineStr">
+        <is>
+          <t>Stability</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="4" t="inlineStr">
+        <is>
+          <t>voters-need-simple-ballots</t>
+        </is>
+      </c>
+      <c r="C482" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D482" s="4" t="inlineStr">
+        <is>
+          <t>Voters need simple ballots and elections they can understand.</t>
+        </is>
+      </c>
+      <c r="M482" s="5" t="inlineStr">
+        <is>
+          <t>Participation</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="4" t="inlineStr">
+        <is>
+          <t>incumbents-major-party-organizations</t>
+        </is>
+      </c>
+      <c r="C483" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="D483" s="4" t="inlineStr">
+        <is>
+          <t>Incumbents and major-party organizations need to protect the rules that protect them, and donors need to protect their channel of influence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="4" t="inlineStr">
+        <is>
+          <t>decade-data-alaska-maine</t>
+        </is>
+      </c>
+      <c r="C484" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D484" s="4" t="inlineStr">
+        <is>
+          <t>A decade of data from Alaska and Maine will show that reformed states elect measurably more median-aligned representatives and that their approval-to-reelection gap narrows compared with matched unreformed states.</t>
+        </is>
+      </c>
+      <c r="G484" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="4" t="inlineStr">
+        <is>
+          <t>legislators-jurisdictions-small-donor</t>
+        </is>
+      </c>
+      <c r="C485" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D485" s="4" t="inlineStr">
+        <is>
+          <t>Legislators in jurisdictions with small-donor matching will track constituent preferences better than legislators in jurisdictions without it.</t>
+        </is>
+      </c>
+      <c r="G485" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="4" t="inlineStr">
+        <is>
+          <t>commission-drawn-maps-will</t>
+        </is>
+      </c>
+      <c r="C486" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D486" s="4" t="inlineStr">
+        <is>
+          <t>Commission-drawn maps will keep producing 15 to 20 percent fewer safe seats than maps drawn by legislatures, cycle after cycle.</t>
+        </is>
+      </c>
+      <c r="G486" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="4" t="inlineStr">
+        <is>
+          <t>jurisdictions-use-ranked-choice</t>
+        </is>
+      </c>
+      <c r="C487" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D487" s="4" t="inlineStr">
+        <is>
+          <t>Jurisdictions that use ranked-choice voting will show persistently lower rates of negative advertising.</t>
+        </is>
+      </c>
+      <c r="G487" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="4" t="inlineStr">
+        <is>
+          <t>reformed-states-will-show</t>
+        </is>
+      </c>
+      <c r="C488" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D488" s="4" t="inlineStr">
+        <is>
+          <t>Reformed states will show no movement on any objective criterion after two full election cycles, or repeal waves will spread beyond single incidents like Burlington.</t>
+        </is>
+      </c>
+      <c r="G488" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="4" t="inlineStr">
+        <is>
+          <t>center-squeeze-other-pathological</t>
+        </is>
+      </c>
+      <c r="C489" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D489" s="4" t="inlineStr">
+        <is>
+          <t>Center-squeeze or other pathological outcomes will recur in ranked-choice elections at rates that measurably erode public trust in results.</t>
+        </is>
+      </c>
+      <c r="G489" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="4" t="inlineStr">
+        <is>
+          <t>representatives-reformed-states-will</t>
+        </is>
+      </c>
+      <c r="C490" s="5" t="inlineStr">
+        <is>
+          <t>claim</t>
+        </is>
+      </c>
+      <c r="D490" s="4" t="inlineStr">
+        <is>
+          <t>Representatives in reformed states will move toward their district medians no faster than representatives in unreformed states.</t>
+        </is>
+      </c>
+      <c r="G490" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AC416"/>
+  <autoFilter ref="A1:AC490"/>
   <dataValidations count="5">
     <dataValidation sqref="C2:C5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"belief,claim,linkage,importance,interest,uniqueness,equivalence,driver,media"</formula1>
@@ -14331,7 +16040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1085"/>
+  <dimension ref="A1:T1166"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -40048,8 +41757,1825 @@
         </is>
       </c>
     </row>
+    <row r="1086">
+      <c r="A1086" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1086" s="5" t="inlineStr">
+        <is>
+          <t>criteria</t>
+        </is>
+      </c>
+      <c r="E1086" s="4" t="inlineStr">
+        <is>
+          <t>Abnormal returns on officials' trades placed before government announcements</t>
+        </is>
+      </c>
+      <c r="T1086" s="4" t="inlineStr">
+        <is>
+          <t>reading: percentage points per year by which officials' portfolios beat or trail a market benchmark, with a separate figure for trades placed shortly before a legislative or regulatory event | validity: Med | reliability: High | linkage: Med | importance: Med | why: Returns are computed from public filings and market prices, so different researchers can reproduce the figure, but the brief's own findings point in opposite directions over different decades, and the linkage dispute asks whether portfolio performance bears on whether ownership creates a voting conflict at all.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1087" s="5" t="inlineStr">
+        <is>
+          <t>criteria</t>
+        </is>
+      </c>
+      <c r="E1087" s="4" t="inlineStr">
+        <is>
+          <t>Share of an official's income sources, debts and foreign ties visible in public filings</t>
+        </is>
+      </c>
+      <c r="T1087" s="4" t="inlineStr">
+        <is>
+          <t>reading: percent of an official's income streams, lenders and foreign income lines that appear in the public record, found by comparing a published tax return against the same official's disclosure form | validity: High | reliability: Med | linkage: High | importance: High | why: It captures exactly what the disclosure-versus-publication argument is about, and the brief says the 2022 release makes a line-by-line comparison possible, but counting what is visible depends on how finely an observer splits income sources and how they treat value ranges against exact figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1088" s="5" t="inlineStr">
+        <is>
+          <t>criteria</t>
+        </is>
+      </c>
+      <c r="E1088" s="4" t="inlineStr">
+        <is>
+          <t>Whether a restriction reaches only the official or also family members who hold no office</t>
+        </is>
+      </c>
+      <c r="T1088" s="4" t="inlineStr">
+        <is>
+          <t>reading: count of people bound by a rule who hold no office (spouses, dependent children, business partners), per rule, and whether the rule reaches them by name or leaves them uncovered | validity: High | reliability: High | linkage: High | importance: High | why: Both sides accept this as the honest test of the anti side's central complaint and of the agree side's substitution worry, since a rule that stops at the official leaves the conflict in spouse accounts and partnerships while a rule that reaches the family binds people who never ran, and reading it requires only the text of the rule.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1089" s="5" t="inlineStr">
+        <is>
+          <t>criteria</t>
+        </is>
+      </c>
+      <c r="E1089" s="4" t="inlineStr">
+        <is>
+          <t>Net worth distribution of candidates and of incoming members before and after a rule takes effect</t>
+        </is>
+      </c>
+      <c r="T1089" s="4" t="inlineStr">
+        <is>
+          <t>reading: median net worth of incoming members and the share whose wealth is in the top 1 percent, from disclosure filings, compared across the cohorts before and after a rule takes effect | validity: Med | reliability: High | linkage: Med | importance: High | why: Disclosure filings give a reproducible figure and it is the yardstick behind the anti side's strongest interest, but candidate wealth moves for many reasons besides ethics rules, so a shift after a rule is suggestive rather than proof that the rule deterred people of ordinary means.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1090" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1090" s="4" t="inlineStr">
+        <is>
+          <t>Official Stock Holdings and Trading Rules</t>
+        </is>
+      </c>
+      <c r="O1090" s="4" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1091" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1091" s="4" t="inlineStr">
+        <is>
+          <t>Family Appointments to Official Roles</t>
+        </is>
+      </c>
+      <c r="O1091" s="4" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1092" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1092" s="4" t="inlineStr">
+        <is>
+          <t>Publication of Officeholders' Tax Returns</t>
+        </is>
+      </c>
+      <c r="O1092" s="4" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+      <c r="B1093" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1093" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1093" s="4" t="inlineStr">
+        <is>
+          <t>tariff-raises-price-good</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+      <c r="B1094" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1094" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1094" s="4" t="inlineStr">
+        <is>
+          <t>other-countries-answer-tariffs</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+      <c r="B1095" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1095" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1095" s="4" t="inlineStr">
+        <is>
+          <t>industries-shielded-foreign-competition</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+      <c r="B1096" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1096" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1096" s="4" t="inlineStr">
+        <is>
+          <t>when-factory-closes-whole</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+      <c r="B1097" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1097" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1097" s="4" t="inlineStr">
+        <is>
+          <t>when-tariff-removed-importers</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="4" t="inlineStr">
+        <is>
+          <t>tariffs-imported-goods-generally</t>
+        </is>
+      </c>
+      <c r="B1098" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1098" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1098" s="4" t="inlineStr">
+        <is>
+          <t>country-lets-its-factories</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+      <c r="B1099" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1099" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1099" s="4" t="inlineStr">
+        <is>
+          <t>country-cannot-make-its</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+      <c r="B1100" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1100" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1100" s="4" t="inlineStr">
+        <is>
+          <t>manufacturing-jobs-offer-steady</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+      <c r="B1101" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1101" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1101" s="4" t="inlineStr">
+        <is>
+          <t>new-industries-need-time</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+      <c r="B1102" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1102" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1102" s="4" t="inlineStr">
+        <is>
+          <t>every-industry-calls-itself</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+      <c r="B1103" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1103" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1103" s="4" t="inlineStr">
+        <is>
+          <t>manufacturers-who-use-protected</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" s="4" t="inlineStr">
+        <is>
+          <t>country-protect-its-key</t>
+        </is>
+      </c>
+      <c r="B1104" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1104" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1104" s="4" t="inlineStr">
+        <is>
+          <t>country-wants-secure-supply</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+      <c r="B1105" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1105" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1105" s="4" t="inlineStr">
+        <is>
+          <t>single-worker-has-almost</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+      <c r="B1106" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1106" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1106" s="4" t="inlineStr">
+        <is>
+          <t>low-paid-workers-spend</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+      <c r="B1107" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1107" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1107" s="4" t="inlineStr">
+        <is>
+          <t>when-wages-too-low</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+      <c r="B1108" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1108" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1108" s="4" t="inlineStr">
+        <is>
+          <t>when-labor-costs-more</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+      <c r="B1109" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1109" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1109" s="4" t="inlineStr">
+        <is>
+          <t>small-businesses-poorer-regions</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" s="4" t="inlineStr">
+        <is>
+          <t>raising-minimum-wage-generally</t>
+        </is>
+      </c>
+      <c r="B1110" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1110" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1110" s="4" t="inlineStr">
+        <is>
+          <t>many-minimum-wage-earners</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+      <c r="B1111" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1111" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1111" s="4" t="inlineStr">
+        <is>
+          <t>employer-who-knows-firing</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+      <c r="B1112" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1112" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1112" s="4" t="inlineStr">
+        <is>
+          <t>small-businesses-cannot-afford</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+      <c r="B1113" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1113" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1113" s="4" t="inlineStr">
+        <is>
+          <t>workers-can-quit-job</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+      <c r="B1114" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1114" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1114" s="4" t="inlineStr">
+        <is>
+          <t>losing-job-can-mean</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+      <c r="B1115" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1115" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1115" s="4" t="inlineStr">
+        <is>
+          <t>workers-who-can-fired</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" s="4" t="inlineStr">
+        <is>
+          <t>employers-generally-free-fire</t>
+        </is>
+      </c>
+      <c r="B1116" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1116" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1116" s="4" t="inlineStr">
+        <is>
+          <t>rules-against-unfair-dismissal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+      <c r="B1117" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1117" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1117" s="4" t="inlineStr">
+        <is>
+          <t>provider-can-slow-down</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+      <c r="B1118" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1118" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1118" s="4" t="inlineStr">
+        <is>
+          <t>many-households-have-little</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+      <c r="B1119" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1119" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1119" s="4" t="inlineStr">
+        <is>
+          <t>new-services-start-small</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+      <c r="B1120" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1120" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1120" s="4" t="inlineStr">
+        <is>
+          <t>all-traffic-alike-live</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+      <c r="B1121" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1121" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1121" s="4" t="inlineStr">
+        <is>
+          <t>building-faster-networks-costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" s="4" t="inlineStr">
+        <is>
+          <t>internet-providers-generally-barred</t>
+        </is>
+      </c>
+      <c r="B1122" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1122" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1122" s="4" t="inlineStr">
+        <is>
+          <t>providers-rarely-block-throttle</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+      <c r="B1123" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1123" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1123" s="4" t="inlineStr">
+        <is>
+          <t>proving-age-means-handing</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+      <c r="B1124" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1124" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1124" s="4" t="inlineStr">
+        <is>
+          <t>teenagers-who-blocked-mainstream</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+      <c r="B1125" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1125" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1125" s="4" t="inlineStr">
+        <is>
+          <t>age-rules-set-law</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+      <c r="B1126" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1126" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1126" s="4" t="inlineStr">
+        <is>
+          <t>society-already-requires-proof</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+      <c r="B1127" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1127" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1127" s="4" t="inlineStr">
+        <is>
+          <t>leaving-choice-parents-has</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" s="4" t="inlineStr">
+        <is>
+          <t>laws-require-people-prove</t>
+        </is>
+      </c>
+      <c r="B1128" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1128" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1128" s="4" t="inlineStr">
+        <is>
+          <t>companies-can-verify-age</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1129" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1129" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1129" s="4" t="inlineStr">
+        <is>
+          <t>partisan-primaries-let-small</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1130" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1130" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1130" s="4" t="inlineStr">
+        <is>
+          <t>gerrymandering-lets-legislators-choose</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1131" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1131" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1131" s="4" t="inlineStr">
+        <is>
+          <t>ranked-choice-voting-produces</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1132" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1132" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1132" s="4" t="inlineStr">
+        <is>
+          <t>campaign-finance-structures-make</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1133" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1133" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1133" s="4" t="inlineStr">
+        <is>
+          <t>third-parties-independents-kept</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1134" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1134" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1134" s="4" t="inlineStr">
+        <is>
+          <t>specific-electoral-reforms-have</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1135" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1135" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1135" s="4" t="inlineStr">
+        <is>
+          <t>two-party-system-has</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1136" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1136" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1136" s="4" t="inlineStr">
+        <is>
+          <t>restoring-voter-s-voice</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1137" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1137" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1137" s="4" t="inlineStr">
+        <is>
+          <t>campaign-finance-restrictions-collide</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1138" s="5" t="inlineStr">
+        <is>
+          <t>argument</t>
+        </is>
+      </c>
+      <c r="C1138" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1138" s="4" t="inlineStr">
+        <is>
+          <t>nonpartisan-primaries-may-weaken</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1139" s="5" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="C1139" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1139" s="4" t="inlineStr">
+        <is>
+          <t>congress-polls-15-25</t>
+        </is>
+      </c>
+      <c r="F1139" s="4" t="inlineStr">
+        <is>
+          <t>Gallup; OpenSecrets, ongoing</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1140" s="5" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="C1140" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1140" s="4" t="inlineStr">
+        <is>
+          <t>primary-voters-measure-significantly</t>
+        </is>
+      </c>
+      <c r="F1140" s="4" t="inlineStr">
+        <is>
+          <t>Pew Research, 2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1141" s="5" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="C1141" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1141" s="4" t="inlineStr">
+        <is>
+          <t>americans-identifying-independents-reached</t>
+        </is>
+      </c>
+      <c r="F1141" s="4" t="inlineStr">
+        <is>
+          <t>Gallup, 2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="1142">
+      <c r="A1142" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1142" s="5" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="C1142" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1142" s="4" t="inlineStr">
+        <is>
+          <t>alaska-s-first-federal</t>
+        </is>
+      </c>
+      <c r="F1142" s="4" t="inlineStr">
+        <is>
+          <t>MIT Election Lab, 2022</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1143" s="5" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="C1143" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1143" s="4" t="inlineStr">
+        <is>
+          <t>independent-redistricting-commissions-arizona</t>
+        </is>
+      </c>
+      <c r="F1143" s="4" t="inlineStr">
+        <is>
+          <t>NCSL, 2021</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1144" s="5" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="C1144" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1144" s="4" t="inlineStr">
+        <is>
+          <t>policy-outcomes-correlate-preferences</t>
+        </is>
+      </c>
+      <c r="F1144" s="4" t="inlineStr">
+        <is>
+          <t>Gilens &amp; Page, Princeton, 2014</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1145" s="5" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="C1145" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1145" s="4" t="inlineStr">
+        <is>
+          <t>burlington-vermont-adopted-ranked</t>
+        </is>
+      </c>
+      <c r="F1145" s="4" t="inlineStr">
+        <is>
+          <t>Burlington city records, 2010</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1146" s="5" t="inlineStr">
+        <is>
+          <t>evidence</t>
+        </is>
+      </c>
+      <c r="C1146" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1146" s="4" t="inlineStr">
+        <is>
+          <t>evidence-whether-nonpartisan-primaries</t>
+        </is>
+      </c>
+      <c r="F1146" s="4" t="inlineStr">
+        <is>
+          <t>NBER working paper</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1147" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="C1147" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1147" s="4" t="inlineStr">
+        <is>
+          <t>independent-voters-about-43</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1148" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="C1148" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1148" s="4" t="inlineStr">
+        <is>
+          <t>voters-need-representatives-who</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1149" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="C1149" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1149" s="4" t="inlineStr">
+        <is>
+          <t>forward-party-other-third</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1150" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="C1150" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1150" s="4" t="inlineStr">
+        <is>
+          <t>opponents-need-governmental-stability</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1151" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="C1151" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1151" s="4" t="inlineStr">
+        <is>
+          <t>voters-need-simple-ballots</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1152" s="5" t="inlineStr">
+        <is>
+          <t>interest</t>
+        </is>
+      </c>
+      <c r="C1152" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1152" s="4" t="inlineStr">
+        <is>
+          <t>incumbents-major-party-organizations</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1153" s="5" t="inlineStr">
+        <is>
+          <t>shared_interest</t>
+        </is>
+      </c>
+      <c r="E1153" s="4" t="inlineStr">
+        <is>
+          <t>Both sides want elections that produce winners most voters can accept as legitimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1154" s="5" t="inlineStr">
+        <is>
+          <t>shared_interest</t>
+        </is>
+      </c>
+      <c r="E1154" s="4" t="inlineStr">
+        <is>
+          <t>Both sides want less political violence and less democratic backsliding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1155" s="5" t="inlineStr">
+        <is>
+          <t>shared_interest</t>
+        </is>
+      </c>
+      <c r="E1155" s="4" t="inlineStr">
+        <is>
+          <t>Both sides want a political system the next generation wants to join.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1156" s="5" t="inlineStr">
+        <is>
+          <t>compromise</t>
+        </is>
+      </c>
+      <c r="E1156" s="4" t="inlineStr">
+        <is>
+          <t>Try reforms at the state level first, and evaluate the Alaska and Maine experiments against the objective criteria before any federal mandate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1157" s="5" t="inlineStr">
+        <is>
+          <t>compromise</t>
+        </is>
+      </c>
+      <c r="E1157" s="4" t="inlineStr">
+        <is>
+          <t>Adopt open primaries without full ranked-choice voting as the first step, so independents can vote while the ballot format stays familiar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1158" s="5" t="inlineStr">
+        <is>
+          <t>compromise</t>
+        </is>
+      </c>
+      <c r="E1158" s="4" t="inlineStr">
+        <is>
+          <t>Use bipartisan redistricting commissions with neutral tiebreakers, on the Colorado model, which both parties have accepted as legitimate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1159" s="5" t="inlineStr">
+        <is>
+          <t>compromise</t>
+        </is>
+      </c>
+      <c r="E1159" s="4" t="inlineStr">
+        <is>
+          <t>Use small-donor matching, like New York City's 8-to-1 model, which amplifies constituent speech rather than restricting anyone's and so avoids the Citizens United problem.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1160" s="5" t="inlineStr">
+        <is>
+          <t>prediction</t>
+        </is>
+      </c>
+      <c r="C1160" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1160" s="4" t="inlineStr">
+        <is>
+          <t>decade-data-alaska-maine</t>
+        </is>
+      </c>
+      <c r="S1160" s="4" t="inlineStr">
+        <is>
+          <t>A decade of Alaska and Maine data</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1161" s="5" t="inlineStr">
+        <is>
+          <t>prediction</t>
+        </is>
+      </c>
+      <c r="C1161" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1161" s="4" t="inlineStr">
+        <is>
+          <t>legislators-jurisdictions-small-donor</t>
+        </is>
+      </c>
+      <c r="S1161" s="4" t="inlineStr">
+        <is>
+          <t>Roll-call alignment studies</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1162" s="5" t="inlineStr">
+        <is>
+          <t>prediction</t>
+        </is>
+      </c>
+      <c r="C1162" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1162" s="4" t="inlineStr">
+        <is>
+          <t>commission-drawn-maps-will</t>
+        </is>
+      </c>
+      <c r="S1162" s="4" t="inlineStr">
+        <is>
+          <t>Each redistricting cycle; Cook ratings, NCSL tracking</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1163" s="5" t="inlineStr">
+        <is>
+          <t>prediction</t>
+        </is>
+      </c>
+      <c r="C1163" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="D1163" s="4" t="inlineStr">
+        <is>
+          <t>jurisdictions-use-ranked-choice</t>
+        </is>
+      </c>
+      <c r="S1163" s="4" t="inlineStr">
+        <is>
+          <t>Ongoing; ad-tone tracking, FairVote and independent replication</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1164" s="5" t="inlineStr">
+        <is>
+          <t>prediction</t>
+        </is>
+      </c>
+      <c r="C1164" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1164" s="4" t="inlineStr">
+        <is>
+          <t>reformed-states-will-show</t>
+        </is>
+      </c>
+      <c r="S1164" s="4" t="inlineStr">
+        <is>
+          <t>Two full election cycles</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1165" s="5" t="inlineStr">
+        <is>
+          <t>prediction</t>
+        </is>
+      </c>
+      <c r="C1165" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1165" s="4" t="inlineStr">
+        <is>
+          <t>center-squeeze-other-pathological</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" s="4" t="inlineStr">
+        <is>
+          <t>we-support-strengthen-democracy</t>
+        </is>
+      </c>
+      <c r="B1166" s="5" t="inlineStr">
+        <is>
+          <t>prediction</t>
+        </is>
+      </c>
+      <c r="C1166" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1166" s="4" t="inlineStr">
+        <is>
+          <t>representatives-reformed-states-will</t>
+        </is>
+      </c>
+      <c r="S1166" s="4" t="inlineStr">
+        <is>
+          <t>5-10 years; roll-call ideal-point estimates by state cohort</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T1085"/>
+  <autoFilter ref="A1:T1166"/>
   <dataValidations count="2">
     <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"argument,assumption,bias,category,cba,common,component,compromise,criteria,criterion,definition,direction,dispute,downstream,engagement,evidence,falsify,impact,interest,interest_listing,law,long_term,media,motive,obstacle,person,prediction,related,rung,shared_interest,short_term,similar,stack,strength,topic_media,topic_values,upstream,value"</formula1>
@@ -40069,7 +43595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F79"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -40243,6 +43769,16 @@
           <t>business-and-economy</t>
         </is>
       </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>Trade covers the buying and selling of goods and services across national borders and the barriers governments place on it.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>favors open trade with few barriers, negative favors tariffs and protection for home industries.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -40260,6 +43796,16 @@
           <t>business-and-economy</t>
         </is>
       </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>Jobs covers pay, hiring, firing and working conditions, and how much of that the law should set.</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>favors stronger legal protections and pay floors for workers, negative favors leaving pay and conditions to employers and the market.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -40311,6 +43857,16 @@
           <t>computers-and-internet</t>
         </is>
       </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>How the internet is run and who sets its rules, from the companies that carry traffic to the laws that govern access, speech and content.</t>
+        </is>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>favors more government rules for how the internet and online platforms operate; negative favors leaving those choices to companies and users.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -41568,8 +45124,140 @@
         </is>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
+        <is>
+          <t>core-principles</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>Core Principles</t>
+        </is>
+      </c>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>society-and-culture</t>
+        </is>
+      </c>
+      <c r="D80" s="5" t="inlineStr">
+        <is>
+          <t>The principles the other positions on this site are argued from.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="4" t="inlineStr">
+        <is>
+          <t>democracy-and-rule-of-law</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Democracy &amp; Rule of Law</t>
+        </is>
+      </c>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>government</t>
+        </is>
+      </c>
+      <c r="D81" s="5" t="inlineStr">
+        <is>
+          <t>How elections, courts and the constitution keep power answerable, and how to strengthen them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="4" t="inlineStr">
+        <is>
+          <t>rights-and-liberty</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>Rights &amp; Liberty</t>
+        </is>
+      </c>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>government</t>
+        </is>
+      </c>
+      <c r="D82" s="5" t="inlineStr">
+        <is>
+          <t>The freedoms the law protects and the responsibilities that come with them.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="4" t="inlineStr">
+        <is>
+          <t>evidence-and-process</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Evidence &amp; Process</t>
+        </is>
+      </c>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>government</t>
+        </is>
+      </c>
+      <c r="D83" s="5" t="inlineStr">
+        <is>
+          <t>How public decisions should be made: on evidence, with scorecards, and with a view to the wider world.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>energy</t>
+        </is>
+      </c>
+      <c r="B84" s="5" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>business-and-economy</t>
+        </is>
+      </c>
+      <c r="D84" s="5" t="inlineStr">
+        <is>
+          <t>How energy is produced, priced and researched.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>immigration</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Immigration</t>
+        </is>
+      </c>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>government</t>
+        </is>
+      </c>
+      <c r="D85" s="5" t="inlineStr">
+        <is>
+          <t>Who may come to the country, on what terms, and how the rules are enforced.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F79"/>
+  <autoFilter ref="A1:F85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>

</xml_diff>

<commit_message>
Fill the last empty cells of the public office topic page
The final sixteen rows (claim strength, rungs, engagement, a criterion,
related topics and best media) each passed the check against the
beliefs beneath the topic, after repair where one failed first. The
page now has no cell reading "Nothing here yet".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KjnsA5EXCtANSJ7uyuepXy
</commit_message>
<xml_diff>
--- a/tools/static-site/ISE_Data_Entry.xlsx
+++ b/tools/static-site/ISE_Data_Entry.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'pages'!$A$1:$AC$490</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'edges'!$A$1:$T$1166</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'edges'!$A$1:$T$1182</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'topics'!$A$1:$F$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -16040,7 +16040,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T1166"/>
+  <dimension ref="A1:T1182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -43574,8 +43574,395 @@
         </is>
       </c>
     </row>
+    <row r="1167">
+      <c r="A1167" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1167" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1167" s="4" t="inlineStr">
+        <is>
+          <t>Congressional Reversal of Pardons</t>
+        </is>
+      </c>
+      <c r="O1167" s="4" t="inlineStr">
+        <is>
+          <t>child</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1168" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1168" s="4" t="inlineStr">
+        <is>
+          <t>Bribery Statutes</t>
+        </is>
+      </c>
+      <c r="O1168" s="4" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1169" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1169" s="4" t="inlineStr">
+        <is>
+          <t>Lobbying Rules</t>
+        </is>
+      </c>
+      <c r="O1169" s="4" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1170" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1170" s="4" t="inlineStr">
+        <is>
+          <t>Financial Disclosure Rules</t>
+        </is>
+      </c>
+      <c r="O1170" s="4" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1171" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1171" s="4" t="inlineStr">
+        <is>
+          <t>Revolving Door Restrictions</t>
+        </is>
+      </c>
+      <c r="O1171" s="4" t="inlineStr">
+        <is>
+          <t>sibling</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1172" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1172" s="4" t="inlineStr">
+        <is>
+          <t>Ethics Rules as a Deterrent to Public Service</t>
+        </is>
+      </c>
+      <c r="O1172" s="4" t="inlineStr">
+        <is>
+          <t>opposing</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1173" s="5" t="inlineStr">
+        <is>
+          <t>related</t>
+        </is>
+      </c>
+      <c r="E1173" s="4" t="inlineStr">
+        <is>
+          <t>Disclosure Rather Than Prohibition</t>
+        </is>
+      </c>
+      <c r="O1173" s="4" t="inlineStr">
+        <is>
+          <t>opposing</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1174" s="5" t="inlineStr">
+        <is>
+          <t>topic_media</t>
+        </is>
+      </c>
+      <c r="D1174" s="4" t="inlineStr">
+        <is>
+          <t>ziobrowski-cheng-boyd-ziobrowski</t>
+        </is>
+      </c>
+      <c r="T1174" s="4" t="inlineStr">
+        <is>
+          <t>medium: Study | tone: Academic | positivity: +60 | strength: 80 | insight: Senators earned abnormal returns on their stock purchases in the 1990s, which points to a trading advantage tied to the office.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1175" s="5" t="inlineStr">
+        <is>
+          <t>topic_media</t>
+        </is>
+      </c>
+      <c r="D1175" s="4" t="inlineStr">
+        <is>
+          <t>eggers-hainmueller-capitol-losses</t>
+        </is>
+      </c>
+      <c r="T1175" s="4" t="inlineStr">
+        <is>
+          <t>medium: Study | tone: Academic | positivity: -50 | strength: 80 | insight: Congressional portfolios did not beat the market, which is hard to square with a systematic insider advantage for a ban to remove.</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1176" s="5" t="inlineStr">
+        <is>
+          <t>strength</t>
+        </is>
+      </c>
+      <c r="C1176" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="E1176" s="4" t="inlineStr">
+        <is>
+          <t>Some new rules on what officeholders may own or trade tend to deter capable people of ordinary means from serving while catching few conflicts the disclosure form did not already show.</t>
+        </is>
+      </c>
+      <c r="O1176" s="4" t="inlineStr">
+        <is>
+          <t>Modest</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1177" s="5" t="inlineStr">
+        <is>
+          <t>strength</t>
+        </is>
+      </c>
+      <c r="C1177" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1177" s="4" t="inlineStr">
+        <is>
+          <t>forced-divestiture-imposes-real</t>
+        </is>
+      </c>
+      <c r="O1177" s="4" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1178" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1178" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="D1178" s="4" t="inlineStr">
+        <is>
+          <t>members-keep-property-rights</t>
+        </is>
+      </c>
+      <c r="O1178" s="4" t="inlineStr">
+        <is>
+          <t>A.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1179" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1179" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="E1179" s="4" t="inlineStr">
+        <is>
+          <t>When the mandatory audit of a president's returns goes dormant, the fix is to hold the IRS to that audit on a deadline and report when it is completed, not to publish the president's tax return.</t>
+        </is>
+      </c>
+      <c r="O1179" s="4" t="inlineStr">
+        <is>
+          <t>C.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1180" s="5" t="inlineStr">
+        <is>
+          <t>rung</t>
+        </is>
+      </c>
+      <c r="C1180" s="5" t="inlineStr">
+        <is>
+          <t>agree</t>
+        </is>
+      </c>
+      <c r="E1180" s="4" t="inlineStr">
+        <is>
+          <t>When a spouse's or business partner's money appears on an officeholder's tax return, it is part of the financial entanglement voters need to see, so publishing it is a privacy cost worth paying rather than a reason to keep the return private.</t>
+        </is>
+      </c>
+      <c r="O1180" s="4" t="inlineStr">
+        <is>
+          <t>C.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1181" s="5" t="inlineStr">
+        <is>
+          <t>engagement</t>
+        </is>
+      </c>
+      <c r="C1181" s="5" t="inlineStr">
+        <is>
+          <t>disagree</t>
+        </is>
+      </c>
+      <c r="E1181" s="4" t="inlineStr">
+        <is>
+          <t>An officeholder who, after a holdings ban or a publication requirement is enacted, openly announces that they will keep their holdings or withhold their returns because the rule reaches lawful property and a family that never ran, and accepts whatever penalty or sanction follows rather than comply quietly.</t>
+        </is>
+      </c>
+      <c r="O1181" s="4" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="T1181" s="4" t="inlineStr">
+        <is>
+          <t>example: defiant officeholder</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" s="4" t="inlineStr">
+        <is>
+          <t>public-office-private-gain</t>
+        </is>
+      </c>
+      <c r="B1182" s="5" t="inlineStr">
+        <is>
+          <t>criteria</t>
+        </is>
+      </c>
+      <c r="E1182" s="4" t="inlineStr">
+        <is>
+          <t>Share of official decisions made by an official holding a personal financial stake in the outcome</t>
+        </is>
+      </c>
+      <c r="T1182" s="4" t="inlineStr">
+        <is>
+          <t>reading: percent of committee votes, rulings or clemency grants in a year where the deciding official or a family member held a stake in the outcome, from disclosure filings matched against the decisions | validity: High | reliability: Med | linkage: High | importance: High | why: It measures the conflict itself rather than a proxy for it, and it is the yardstick behind an interest cited on every belief page in the topic, but building the reading requires matching holdings against decisions, and no matched study of members' holdings against their roll-call votes yet exists, so observers will draw the line between stake and no stake differently.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:T1166"/>
+  <autoFilter ref="A1:T1182"/>
   <dataValidations count="2">
     <dataValidation sqref="B2:B5000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"argument,assumption,bias,category,cba,common,component,compromise,criteria,criterion,definition,direction,dispute,downstream,engagement,evidence,falsify,impact,interest,interest_listing,law,long_term,media,motive,obstacle,person,prediction,related,rung,shared_interest,short_term,similar,stack,strength,topic_media,topic_values,upstream,value"</formula1>

</xml_diff>